<commit_message>
Regen CPL_Data.js + xlsx exports from local generator run
Timestamp refresh only — daily workflow will re-overwrite these tomorrow.
Committed to keep the working tree clean alongside the structural change.

https://claude.ai/code/session_018pUUHRb3yZXrDWJG7p2Kci
</commit_message>
<xml_diff>
--- a/exports/exhibit-by-college.xlsx
+++ b/exports/exhibit-by-college.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Credit Recommendations by Colle" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Credit Recommendations by Colle" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Daily regen side-effects from local excel_to_dashboard.py run (Session 5a)
</commit_message>
<xml_diff>
--- a/exports/exhibit-by-college.xlsx
+++ b/exports/exhibit-by-college.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Credit Recommendations by Colle" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Credit Recommendations by Colle" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H103"/>
+  <dimension ref="A1:H104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -507,7 +507,7 @@
         <v>163</v>
       </c>
       <c r="H2" t="n">
-        <v>5</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="3">
@@ -520,22 +520,22 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>428</v>
+        <v>447</v>
       </c>
       <c r="D3" t="n">
-        <v>310</v>
+        <v>319</v>
       </c>
       <c r="E3" t="n">
         <v>20</v>
       </c>
       <c r="F3" t="n">
-        <v>135</v>
+        <v>149</v>
       </c>
       <c r="G3" t="n">
-        <v>170</v>
+        <v>189</v>
       </c>
       <c r="H3" t="n">
-        <v>4</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="4">
@@ -548,10 +548,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>392</v>
+        <v>414</v>
       </c>
       <c r="D4" t="n">
-        <v>331</v>
+        <v>353</v>
       </c>
       <c r="E4" t="n">
         <v>18</v>
@@ -563,7 +563,7 @@
         <v>78</v>
       </c>
       <c r="H4" t="n">
-        <v>3.6</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="5">
@@ -591,7 +591,7 @@
         <v>74</v>
       </c>
       <c r="H5" t="n">
-        <v>3.1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -604,10 +604,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D6" t="n">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E6" t="n">
         <v>15</v>
@@ -616,10 +616,10 @@
         <v>11</v>
       </c>
       <c r="G6" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H6" t="n">
-        <v>2.9</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="7">
@@ -647,7 +647,7 @@
         <v>202</v>
       </c>
       <c r="H7" t="n">
-        <v>2.9</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="8">
@@ -703,7 +703,7 @@
         <v>20</v>
       </c>
       <c r="H9" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="10">
@@ -731,7 +731,7 @@
         <v>202</v>
       </c>
       <c r="H10" t="n">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="11">
@@ -768,23 +768,23 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Bakersfield College</t>
+          <t>San Bernardino Valley College</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>224</v>
+        <v>236</v>
       </c>
       <c r="D12" t="n">
-        <v>117</v>
+        <v>133</v>
       </c>
       <c r="E12" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="F12" t="n">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="G12" t="n">
-        <v>153</v>
+        <v>84</v>
       </c>
       <c r="H12" t="n">
         <v>2.1</v>
@@ -796,23 +796,23 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Cabrillo College</t>
+          <t>Bakersfield College</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="D13" t="n">
-        <v>167</v>
+        <v>117</v>
       </c>
       <c r="E13" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="F13" t="n">
-        <v>32</v>
+        <v>90</v>
       </c>
       <c r="G13" t="n">
-        <v>99</v>
+        <v>153</v>
       </c>
       <c r="H13" t="n">
         <v>2</v>
@@ -824,26 +824,26 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Clovis Community College</t>
+          <t>Cabrillo College</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>198</v>
+        <v>219</v>
       </c>
       <c r="D14" t="n">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="E14" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="F14" t="n">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="G14" t="n">
-        <v>8</v>
+        <v>99</v>
       </c>
       <c r="H14" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -852,23 +852,23 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>West Los Angeles College</t>
+          <t>Clovis Community College</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="D15" t="n">
-        <v>77</v>
+        <v>161</v>
       </c>
       <c r="E15" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G15" t="n">
-        <v>125</v>
+        <v>8</v>
       </c>
       <c r="H15" t="n">
         <v>1.8</v>
@@ -880,23 +880,23 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Santiago Canyon College</t>
+          <t>Los Angeles Trade Technical College</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="D16" t="n">
-        <v>9</v>
+        <v>177</v>
       </c>
       <c r="E16" t="n">
+        <v>6</v>
+      </c>
+      <c r="F16" t="n">
         <v>1</v>
       </c>
-      <c r="F16" t="n">
-        <v>0</v>
-      </c>
       <c r="G16" t="n">
-        <v>189</v>
+        <v>53</v>
       </c>
       <c r="H16" t="n">
         <v>1.8</v>
@@ -908,26 +908,26 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Los Angeles Trade Technical College</t>
+          <t>West Los Angeles College</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>187</v>
+        <v>194</v>
       </c>
       <c r="D17" t="n">
-        <v>174</v>
+        <v>77</v>
       </c>
       <c r="E17" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F17" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="G17" t="n">
-        <v>53</v>
+        <v>125</v>
       </c>
       <c r="H17" t="n">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="18">
@@ -936,23 +936,23 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Merced College</t>
+          <t>Santiago Canyon College</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="D18" t="n">
-        <v>142</v>
+        <v>9</v>
       </c>
       <c r="E18" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>42</v>
+        <v>189</v>
       </c>
       <c r="H18" t="n">
         <v>1.7</v>
@@ -964,23 +964,23 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>San Bernardino Valley College</t>
+          <t>Merced College</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="D19" t="n">
-        <v>126</v>
+        <v>142</v>
       </c>
       <c r="E19" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F19" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G19" t="n">
-        <v>84</v>
+        <v>42</v>
       </c>
       <c r="H19" t="n">
         <v>1.7</v>
@@ -1011,7 +1011,7 @@
         <v>105</v>
       </c>
       <c r="H20" t="n">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="21">
@@ -1024,10 +1024,10 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D21" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E21" t="n">
         <v>12</v>
@@ -1048,26 +1048,26 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Los Angeles Valley College</t>
+          <t>Los Angeles Mission College</t>
         </is>
       </c>
       <c r="C22" t="n">
         <v>159</v>
       </c>
       <c r="D22" t="n">
-        <v>85</v>
+        <v>101</v>
       </c>
       <c r="E22" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G22" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="H22" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="23">
@@ -1076,23 +1076,23 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>San Diego Mesa College</t>
+          <t>Los Angeles Valley College</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="D23" t="n">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="E23" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="F23" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H23" t="n">
         <v>1.4</v>
@@ -1104,23 +1104,23 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Barstow Community College</t>
+          <t>San Diego Mesa College</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="D24" t="n">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E24" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="F24" t="n">
-        <v>90</v>
+        <v>3</v>
       </c>
       <c r="G24" t="n">
-        <v>88</v>
+        <v>6</v>
       </c>
       <c r="H24" t="n">
         <v>1.4</v>
@@ -1132,26 +1132,26 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Coastline Community College</t>
+          <t>Barstow Community College</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D25" t="n">
-        <v>139</v>
+        <v>94</v>
       </c>
       <c r="E25" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="F25" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="G25" t="n">
-        <v>0</v>
+        <v>88</v>
       </c>
       <c r="H25" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="26">
@@ -1160,23 +1160,23 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>San Diego City College</t>
+          <t>Coastline Community College</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="D26" t="n">
-        <v>102</v>
+        <v>139</v>
       </c>
       <c r="E26" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F26" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="G26" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H26" t="n">
         <v>1.3</v>
@@ -1188,23 +1188,23 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Lake Tahoe Community College</t>
+          <t>San Diego City College</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="D27" t="n">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E27" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="F27" t="n">
-        <v>46</v>
+        <v>12</v>
       </c>
       <c r="G27" t="n">
-        <v>66</v>
+        <v>22</v>
       </c>
       <c r="H27" t="n">
         <v>1.3</v>
@@ -1216,23 +1216,23 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Glendale Community College</t>
+          <t>Lake Tahoe Community College</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="D28" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="E28" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="F28" t="n">
-        <v>17</v>
+        <v>46</v>
       </c>
       <c r="G28" t="n">
-        <v>23</v>
+        <v>66</v>
       </c>
       <c r="H28" t="n">
         <v>1.2</v>
@@ -1244,26 +1244,26 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>San Jose City College</t>
+          <t>Glendale Community College</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="D29" t="n">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="E29" t="n">
         <v>14</v>
       </c>
       <c r="F29" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="G29" t="n">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="H29" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="30">
@@ -1272,26 +1272,26 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>De Anza College</t>
+          <t>San Jose City College</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="D30" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E30" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="F30" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="G30" t="n">
-        <v>59</v>
+        <v>12</v>
       </c>
       <c r="H30" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="31">
@@ -1300,26 +1300,26 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Las Positas College</t>
+          <t>De Anza College</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="D31" t="n">
-        <v>87</v>
+        <v>102</v>
       </c>
       <c r="E31" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F31" t="n">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="G31" t="n">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="H31" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="32">
@@ -1328,23 +1328,23 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Foothill College</t>
+          <t>Las Positas College</t>
         </is>
       </c>
       <c r="C32" t="n">
         <v>112</v>
       </c>
       <c r="D32" t="n">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E32" t="n">
         <v>10</v>
       </c>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="G32" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="H32" t="n">
         <v>1</v>
@@ -1356,23 +1356,23 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Chabot College</t>
+          <t>Foothill College</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D33" t="n">
-        <v>71</v>
+        <v>103</v>
       </c>
       <c r="E33" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F33" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="G33" t="n">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="H33" t="n">
         <v>1</v>
@@ -1384,23 +1384,23 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Solano Community College</t>
+          <t>Chabot College</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D34" t="n">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="E34" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F34" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="G34" t="n">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="H34" t="n">
         <v>1</v>
@@ -1412,23 +1412,23 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Reedley College</t>
+          <t>Solano Community College</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D35" t="n">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="E35" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F35" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="G35" t="n">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="H35" t="n">
         <v>1</v>
@@ -1440,23 +1440,23 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Woodland Community College</t>
+          <t>Reedley College</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="D36" t="n">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="E36" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="F36" t="n">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="G36" t="n">
-        <v>11</v>
+        <v>41</v>
       </c>
       <c r="H36" t="n">
         <v>1</v>
@@ -1468,23 +1468,23 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>College of the Desert</t>
+          <t>Santa Monica College</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D37" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E37" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F37" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="G37" t="n">
-        <v>76</v>
+        <v>53</v>
       </c>
       <c r="H37" t="n">
         <v>1</v>
@@ -1496,26 +1496,26 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Santa Monica College</t>
+          <t>Woodland Community College</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D38" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="E38" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="F38" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="G38" t="n">
-        <v>51</v>
+        <v>11</v>
       </c>
       <c r="H38" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="39">
@@ -1524,23 +1524,23 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Napa Valley College</t>
+          <t>College of the Desert</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D39" t="n">
-        <v>86</v>
+        <v>54</v>
       </c>
       <c r="E39" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="F39" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="G39" t="n">
-        <v>19</v>
+        <v>76</v>
       </c>
       <c r="H39" t="n">
         <v>0.9</v>
@@ -1556,10 +1556,10 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D40" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E40" t="n">
         <v>5</v>
@@ -1568,7 +1568,7 @@
         <v>12</v>
       </c>
       <c r="G40" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="H40" t="n">
         <v>0.9</v>
@@ -1580,23 +1580,23 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Ventura College</t>
+          <t>Napa Valley College</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D41" t="n">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="E41" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F41" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G41" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="H41" t="n">
         <v>0.9</v>
@@ -1608,23 +1608,23 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Sierra College</t>
+          <t>Ventura College</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D42" t="n">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="E42" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="F42" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="G42" t="n">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="H42" t="n">
         <v>0.9</v>
@@ -1636,23 +1636,23 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Cypress College</t>
+          <t>Sierra College</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="D43" t="n">
-        <v>86</v>
+        <v>66</v>
       </c>
       <c r="E43" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="F43" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="G43" t="n">
-        <v>1</v>
+        <v>46</v>
       </c>
       <c r="H43" t="n">
         <v>0.9</v>
@@ -1664,26 +1664,26 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>College of the Sequoias</t>
+          <t>Cypress College</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="D44" t="n">
-        <v>60</v>
+        <v>87</v>
       </c>
       <c r="E44" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="F44" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="G44" t="n">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="H44" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="45">
@@ -1692,23 +1692,23 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Mendocino College</t>
+          <t>College of the Sequoias</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D45" t="n">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="E45" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F45" t="n">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="G45" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="H45" t="n">
         <v>0.8</v>
@@ -1724,10 +1724,10 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="D46" t="n">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="E46" t="n">
         <v>5</v>
@@ -1736,10 +1736,10 @@
         <v>6</v>
       </c>
       <c r="G46" t="n">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="H46" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="47">
@@ -1748,26 +1748,26 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Cuesta College</t>
+          <t>Mendocino College</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="D47" t="n">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="E47" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F47" t="n">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="G47" t="n">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="H47" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="48">
@@ -1776,23 +1776,23 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>CA MAP INITIATIVE COLLEGE</t>
+          <t>Cerritos College</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="D48" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E48" t="n">
         <v>5</v>
       </c>
       <c r="F48" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G48" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H48" t="n">
         <v>0.7</v>
@@ -1804,20 +1804,20 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>East Los Angeles College</t>
+          <t>Cuesta College</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D49" t="n">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="E49" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F49" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="G49" t="n">
         <v>11</v>
@@ -1832,23 +1832,23 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Columbia College</t>
+          <t>East Los Angeles College</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D50" t="n">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="E50" t="n">
         <v>5</v>
       </c>
       <c r="F50" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="G50" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="H50" t="n">
         <v>0.7</v>
@@ -1860,23 +1860,23 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Madera College</t>
+          <t>CA MAP INITIATIVE COLLEGE</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D51" t="n">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="E51" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="F51" t="n">
         <v>2</v>
       </c>
       <c r="G51" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H51" t="n">
         <v>0.7</v>
@@ -1888,23 +1888,23 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Cerritos College</t>
+          <t>Columbia College</t>
         </is>
       </c>
       <c r="C52" t="n">
         <v>73</v>
       </c>
       <c r="D52" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E52" t="n">
         <v>5</v>
       </c>
       <c r="F52" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="G52" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H52" t="n">
         <v>0.7</v>
@@ -1916,23 +1916,23 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Contra Costa College</t>
+          <t>Madera College</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="D53" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E53" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="F53" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="G53" t="n">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="H53" t="n">
         <v>0.7</v>
@@ -1944,23 +1944,23 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Los Angeles Mission College</t>
+          <t>Contra Costa College</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D54" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="E54" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F54" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="G54" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="H54" t="n">
         <v>0.6</v>
@@ -2336,7 +2336,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Mt. San Antonio College</t>
+          <t>Yuba College</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -2352,7 +2352,7 @@
         <v>0</v>
       </c>
       <c r="G68" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H68" t="n">
         <v>0.5</v>
@@ -2364,7 +2364,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Yuba College</t>
+          <t>Mt. San Antonio College</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -2380,7 +2380,7 @@
         <v>0</v>
       </c>
       <c r="G69" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H69" t="n">
         <v>0.5</v>
@@ -2448,14 +2448,14 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>College of the Redwoods</t>
+          <t>Folsom Lake College</t>
         </is>
       </c>
       <c r="C72" t="n">
         <v>53</v>
       </c>
       <c r="D72" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E72" t="n">
         <v>3</v>
@@ -2476,14 +2476,14 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Folsom Lake College</t>
+          <t>College of the Redwoods</t>
         </is>
       </c>
       <c r="C73" t="n">
         <v>53</v>
       </c>
       <c r="D73" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E73" t="n">
         <v>3</v>
@@ -2504,7 +2504,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Victor Valley College</t>
+          <t>El Camino College</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -2560,7 +2560,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Diablo Valley College</t>
+          <t>Santa Rosa Junior College</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -2588,7 +2588,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>El Camino College</t>
+          <t>Ohlone College</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -2616,7 +2616,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Golden West College</t>
+          <t>Victor Valley College</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -2644,7 +2644,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Los Angeles City College</t>
+          <t>Sacramento City College</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Ohlone College</t>
+          <t>Golden West College</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -2700,7 +2700,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Oxnard College</t>
+          <t>Diablo Valley College</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -2756,7 +2756,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Sacramento City College</t>
+          <t>West Valley College</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -2784,7 +2784,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Santa Rosa Junior College</t>
+          <t>Los Angeles City College</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -2812,7 +2812,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Coalinga College</t>
+          <t>Oxnard College</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -2840,7 +2840,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>West Valley College</t>
+          <t>Coalinga College</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -2900,10 +2900,10 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D88" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E88" t="n">
         <v>3</v>
@@ -2912,7 +2912,7 @@
         <v>15</v>
       </c>
       <c r="G88" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H88" t="n">
         <v>0.3</v>
@@ -2928,10 +2928,10 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D89" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E89" t="n">
         <v>5</v>
@@ -2940,7 +2940,7 @@
         <v>14</v>
       </c>
       <c r="G89" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H89" t="n">
         <v>0.3</v>
@@ -3008,26 +3008,26 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Cerro Coso Community College</t>
+          <t>Los Angeles Southwest College</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="D92" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F92" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="G92" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H92" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="93">
@@ -3036,23 +3036,23 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Mission College</t>
+          <t>Cerro Coso Community College</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D93" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="E93" t="n">
         <v>3</v>
       </c>
       <c r="F93" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="G93" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H93" t="n">
         <v>0.1</v>
@@ -3064,23 +3064,23 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Lassen College</t>
+          <t>Mission College</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D94" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E94" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F94" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="G94" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="H94" t="n">
         <v>0.1</v>
@@ -3120,23 +3120,23 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Grossmont College</t>
+          <t>Lassen College</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D96" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E96" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F96" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G96" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H96" t="n">
         <v>0.1</v>
@@ -3148,23 +3148,23 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Los Angeles Harbor College</t>
+          <t>Grossmont College</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D97" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E97" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F97" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G97" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="H97" t="n">
         <v>0.1</v>
@@ -3176,23 +3176,23 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Skyline College</t>
+          <t>Los Angeles Harbor College</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D98" t="n">
+        <v>9</v>
+      </c>
+      <c r="E98" t="n">
+        <v>3</v>
+      </c>
+      <c r="F98" t="n">
         <v>1</v>
       </c>
-      <c r="E98" t="n">
-        <v>1</v>
-      </c>
-      <c r="F98" t="n">
-        <v>0</v>
-      </c>
       <c r="G98" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="H98" t="n">
         <v>0.1</v>
@@ -3204,11 +3204,11 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>College of San Mateo</t>
+          <t>Skyline College</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D99" t="n">
         <v>1</v>
@@ -3220,7 +3220,7 @@
         <v>0</v>
       </c>
       <c r="G99" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H99" t="n">
         <v>0.1</v>
@@ -3232,26 +3232,26 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Orange Coast College</t>
+          <t>College of San Mateo</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D100" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E100" t="n">
         <v>1</v>
       </c>
       <c r="F100" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G100" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H100" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="101">
@@ -3260,23 +3260,23 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Santa Barbara City College</t>
+          <t>Orange Coast College</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D101" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E101" t="n">
         <v>1</v>
       </c>
       <c r="F101" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G101" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H101" t="n">
         <v>0</v>
@@ -3288,52 +3288,80 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
+          <t>Santa Barbara City College</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>2</v>
+      </c>
+      <c r="D102" t="n">
+        <v>2</v>
+      </c>
+      <c r="E102" t="n">
+        <v>1</v>
+      </c>
+      <c r="F102" t="n">
+        <v>0</v>
+      </c>
+      <c r="G102" t="n">
+        <v>2</v>
+      </c>
+      <c r="H102" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>102</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
           <t>Southwestern College</t>
         </is>
       </c>
-      <c r="C102" t="n">
-        <v>2</v>
-      </c>
-      <c r="D102" t="n">
+      <c r="C103" t="n">
+        <v>2</v>
+      </c>
+      <c r="D103" t="n">
         <v>1</v>
       </c>
-      <c r="E102" t="n">
-        <v>2</v>
-      </c>
-      <c r="F102" t="n">
-        <v>0</v>
-      </c>
-      <c r="G102" t="n">
-        <v>0</v>
-      </c>
-      <c r="H102" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
+      <c r="E103" t="n">
+        <v>2</v>
+      </c>
+      <c r="F103" t="n">
+        <v>0</v>
+      </c>
+      <c r="G103" t="n">
+        <v>0</v>
+      </c>
+      <c r="H103" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>101 colleges</t>
-        </is>
-      </c>
-      <c r="C103" t="n">
-        <v>10683</v>
-      </c>
-      <c r="D103" t="n">
-        <v>7953</v>
-      </c>
-      <c r="F103" t="n">
-        <v>1151</v>
-      </c>
-      <c r="G103" t="n">
-        <v>3084</v>
-      </c>
-      <c r="H103" t="n">
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>102 colleges</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>10928</v>
+      </c>
+      <c r="D104" t="n">
+        <v>8077</v>
+      </c>
+      <c r="F104" t="n">
+        <v>1160</v>
+      </c>
+      <c r="G104" t="n">
+        <v>3137</v>
+      </c>
+      <c r="H104" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>